<commit_message>
Switched Abi 8h event req for friendship level req
</commit_message>
<xml_diff>
--- a/Notes/AdvAbigail Tracker.xlsx
+++ b/Notes/AdvAbigail Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Si\Gen\SDV Projects\Posted\Adventurer Abigail\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programs\Steam\Steam\steamapps\common\Stardew Valley\SiMods\[Si]\AdvAbigail\Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BBFFCB1-AF54-4E45-8AF5-6F3D2BE21C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B4D206-A99D-4457-8881-3CDAAA4D4698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="152">
   <si>
     <t>ID</t>
   </si>
@@ -477,6 +477,21 @@
   </si>
   <si>
     <t>Marlon takes a vacay - start guildweek here</t>
+  </si>
+  <si>
+    <t>AdvAbiWiz</t>
+  </si>
+  <si>
+    <t>Scene of her parents being concerned</t>
+  </si>
+  <si>
+    <t>xover w bearfam - buys some supplies from gunnar for a mine run</t>
+  </si>
+  <si>
+    <t>Arc 3</t>
+  </si>
+  <si>
+    <t>AdvAbiDwarf</t>
   </si>
 </sst>
 </file>
@@ -500,7 +515,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -555,6 +570,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -568,7 +589,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -579,6 +600,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -864,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W45"/>
+  <dimension ref="A1:W47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" customWidth="1"/>
@@ -1089,6 +1111,9 @@
       <c r="F8">
         <v>0</v>
       </c>
+      <c r="I8" t="s">
+        <v>147</v>
+      </c>
       <c r="J8" t="s">
         <v>66</v>
       </c>
@@ -1305,7 +1330,7 @@
       </c>
       <c r="K16" s="3">
         <f>ROUND((SUM(K14,K15)/COUNT(A:A))*100,2)</f>
-        <v>61.9</v>
+        <v>59.09</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.3">
@@ -1496,6 +1521,9 @@
       <c r="I25" t="s">
         <v>139</v>
       </c>
+      <c r="N25" s="10" t="s">
+        <v>146</v>
+      </c>
       <c r="S25" t="s">
         <v>31</v>
       </c>
@@ -1549,13 +1577,19 @@
       <c r="A28">
         <v>262213026</v>
       </c>
+      <c r="C28" s="4"/>
       <c r="D28" t="s">
         <v>86</v>
       </c>
       <c r="F28">
         <v>10</v>
       </c>
-      <c r="H28" s="5"/>
+      <c r="H28" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="I28" t="s">
+        <v>151</v>
+      </c>
       <c r="S28" s="4" t="s">
         <v>78</v>
       </c>
@@ -1564,6 +1598,7 @@
       <c r="A29">
         <v>262213027</v>
       </c>
+      <c r="C29" s="4"/>
       <c r="D29" t="s">
         <v>33</v>
       </c>
@@ -1581,10 +1616,11 @@
       <c r="A30">
         <v>262213028</v>
       </c>
+      <c r="C30" s="4"/>
       <c r="D30" t="s">
         <v>34</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="H30" s="7" t="s">
         <v>94</v>
       </c>
       <c r="S30" s="4" t="s">
@@ -1598,8 +1634,9 @@
       <c r="A31">
         <v>262213029</v>
       </c>
+      <c r="C31" s="4"/>
       <c r="D31" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="S31" t="s">
         <v>36</v>
@@ -1609,6 +1646,7 @@
       <c r="A32">
         <v>262213030</v>
       </c>
+      <c r="C32" s="4"/>
       <c r="D32" t="s">
         <v>61</v>
       </c>
@@ -1620,6 +1658,7 @@
       <c r="A33">
         <v>262213031</v>
       </c>
+      <c r="C33" s="4"/>
       <c r="D33" t="s">
         <v>57</v>
       </c>
@@ -1631,6 +1670,7 @@
       <c r="A34">
         <v>262213032</v>
       </c>
+      <c r="C34" s="4"/>
       <c r="D34" t="s">
         <v>130</v>
       </c>
@@ -1642,6 +1682,7 @@
       <c r="A35">
         <v>262213033</v>
       </c>
+      <c r="C35" s="4"/>
       <c r="D35" t="s">
         <v>144</v>
       </c>
@@ -1653,6 +1694,7 @@
       <c r="A36">
         <v>262213034</v>
       </c>
+      <c r="C36" s="4"/>
       <c r="D36" t="s">
         <v>131</v>
       </c>
@@ -1664,13 +1706,7 @@
       <c r="A37">
         <v>262213035</v>
       </c>
-      <c r="D37" t="s">
-        <v>56</v>
-      </c>
-      <c r="E37" t="s">
-        <v>27</v>
-      </c>
-      <c r="H37" s="5"/>
+      <c r="C37" s="4"/>
       <c r="S37" t="s">
         <v>43</v>
       </c>
@@ -1683,8 +1719,12 @@
         <v>262213036</v>
       </c>
       <c r="D38" t="s">
-        <v>45</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="E38" t="s">
+        <v>27</v>
+      </c>
+      <c r="H38" s="5"/>
       <c r="S38" t="s">
         <v>75</v>
       </c>
@@ -1697,7 +1737,7 @@
         <v>262213037</v>
       </c>
       <c r="D39" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.3">
@@ -1705,7 +1745,7 @@
         <v>262213038</v>
       </c>
       <c r="D40" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="S40" t="s">
         <v>48</v>
@@ -1716,7 +1756,7 @@
         <v>262213039</v>
       </c>
       <c r="D41" t="s">
-        <v>132</v>
+        <v>44</v>
       </c>
       <c r="S41" t="s">
         <v>49</v>
@@ -1727,7 +1767,7 @@
         <v>262213040</v>
       </c>
       <c r="D42" t="s">
-        <v>59</v>
+        <v>132</v>
       </c>
       <c r="S42" t="s">
         <v>50</v>
@@ -1738,23 +1778,39 @@
         <v>262213041</v>
       </c>
       <c r="D43" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="S43" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>262213042</v>
+      </c>
       <c r="D44" t="s">
-        <v>137</v>
+        <v>46</v>
       </c>
       <c r="S44" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="H45" s="7" t="s">
+      <c r="A45">
+        <v>262213043</v>
+      </c>
+      <c r="D45" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="H46" s="7" t="s">
         <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="O47" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>